<commit_message>
Docs | 회원 관련 테이블 추가, 엑셀 문서 수정 | add table related with member, update excel file
</commit_message>
<xml_diff>
--- a/FuntionalSpecification.xlsx
+++ b/FuntionalSpecification.xlsx
@@ -9,12 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25610" windowHeight="12050" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25610" windowHeight="12050" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet6" sheetId="8" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="7" r:id="rId4"/>
     <sheet name="Sheet4" sheetId="6" r:id="rId5"/>
     <sheet name="히스토리" sheetId="5" r:id="rId6"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="282">
   <si>
     <t>기능 정의서</t>
   </si>
@@ -154,55 +154,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>객체ERP 느낌</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>생성일시</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>수정일시</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>삭제 여부(바로 delete 안하고 조금 남겨놓기위해)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>기능명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>작업 요소</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>구현 대상</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>기능 정의</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>공통</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>pc</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>mobile</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>웹</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>개발</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1096,6 +1048,122 @@
   </si>
   <si>
     <t>웹상에서의 행동과 현실에서의 행동 or 객체를 기준으로</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기능 명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기능 코드</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>깊이 1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>깊이 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>깊이 3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기능 설명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사이트 목록 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>카테고리별 사이트 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>관리자용 사이트 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>검색 사이트 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>화면에 요청사항에 맞는 사이트 목록 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>카테고리 목록 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이용자용 카테고리 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>관리자용 카테고리 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>중요도</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>진행 단계</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>화면에 요청사항에 맞는 카테고리 목록 출력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>구현 대상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조회수 증가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이용자가 사이트 클릭 시 조회수 증가</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>싫어요 증가/ 감소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>좋아요 증가 / 감소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이용자가 사이트 싫어요 클릭 시 수 증가/ 감소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이용자가 사이트 좋아요 클릭 시 수 증가/ 다시 클릭하면 다시 감소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>회원 정보 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>관리자용 회원정보 리스트 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>관리자용 회원정보 세부 조회</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이용자용 회원정보 세부 조회</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1258,15 +1326,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
@@ -1340,7 +1405,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1762,18 +1827,18 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="D24" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="D25" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E25" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
@@ -1814,13 +1879,13 @@
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E50" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1832,84 +1897,656 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G124"/>
+  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.08203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.08203125" customWidth="1"/>
-    <col min="7" max="7" width="7.58203125" customWidth="1"/>
-    <col min="8" max="9" width="6.75" customWidth="1"/>
-    <col min="12" max="12" width="40.25" customWidth="1"/>
+    <col min="1" max="1" width="8.58203125" style="6"/>
+    <col min="2" max="2" width="22.5" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.08203125" style="16" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5" style="6" customWidth="1"/>
+    <col min="6" max="6" width="48.08203125" style="8" customWidth="1"/>
+    <col min="7" max="7" width="51" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="8.58203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="D3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="D4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F6" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="F7" s="27"/>
-      <c r="G7" s="2" t="s">
+    <row r="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="4"/>
+      <c r="B1" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" s="19"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="18"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="E2" s="18"/>
+    </row>
+    <row r="4" spans="1:7" ht="17.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="B4" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B5" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="I7" s="2" t="s">
+    </row>
+    <row r="6" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="12"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="12"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="7" customFormat="1" ht="51" x14ac:dyDescent="0.45">
+      <c r="A8" s="12"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="7" customFormat="1" ht="34" x14ac:dyDescent="0.45">
+      <c r="A9" s="12"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="7" customFormat="1" ht="34" x14ac:dyDescent="0.45">
+      <c r="A10" s="12"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="12"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="12"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="12"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="12"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="D14" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="7" customFormat="1" ht="102" x14ac:dyDescent="0.45">
+      <c r="A15" s="12"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="D17" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="D18" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="51" x14ac:dyDescent="0.45">
+      <c r="D20" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="J7" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="K7" s="2" t="s">
+      <c r="E20" s="17" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="22" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="20"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="L7" s="27"/>
-    </row>
-    <row r="10" spans="1:12" ht="21" x14ac:dyDescent="0.45">
-      <c r="C10" s="1"/>
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" s="12"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="12"/>
+      <c r="F22" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="D23" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B25" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="12"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="102" x14ac:dyDescent="0.45">
+      <c r="D27" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B31" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="34" x14ac:dyDescent="0.45">
+      <c r="D32" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="E33" s="17"/>
+    </row>
+    <row r="34" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="12"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="12"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D35" s="16" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="12"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D37" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="C39" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A40" s="12"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E40" s="12"/>
+      <c r="F40" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A41" s="12"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E41" s="12"/>
+      <c r="F41" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A42" s="12"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E42" s="12"/>
+      <c r="F42" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A44" s="12"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E44" s="12"/>
+    </row>
+    <row r="45" spans="1:6" s="7" customFormat="1" ht="85" x14ac:dyDescent="0.45">
+      <c r="A45" s="12"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="C49" s="16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="68" x14ac:dyDescent="0.45">
+      <c r="D50" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F51" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F52" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A54" s="12"/>
+      <c r="B54" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C54" s="14"/>
+      <c r="E54" s="12"/>
+    </row>
+    <row r="55" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A55" s="12"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A57" s="12"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="E57" s="12"/>
+    </row>
+    <row r="58" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A58" s="12"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="B61" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="D62" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="B65" s="16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="B73" s="16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D74" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="F75" s="7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D76" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="E76" s="8"/>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D77" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="E77" s="8"/>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D78" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D79" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="D80" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="B82" s="16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="B94" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="C94" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A95" s="12"/>
+      <c r="B95" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C95" s="14"/>
+      <c r="D95" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E95" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="F95" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A96" s="12"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="14"/>
+      <c r="D96" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E96" s="12"/>
+      <c r="F96" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A97" s="12"/>
+      <c r="B97" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C97" s="14"/>
+      <c r="D97" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E97" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A98" s="12"/>
+      <c r="B98" s="14"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E98" s="12"/>
+      <c r="F98" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="B99" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" s="7" customFormat="1" ht="68" x14ac:dyDescent="0.45">
+      <c r="A107" s="12"/>
+      <c r="B107" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C107" s="14"/>
+      <c r="D107" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E107" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="F107" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A108" s="12"/>
+      <c r="B108" s="14"/>
+      <c r="C108" s="14"/>
+      <c r="E108" s="12"/>
+      <c r="F108" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" s="7" customFormat="1" ht="51" x14ac:dyDescent="0.45">
+      <c r="A114" s="12"/>
+      <c r="B114" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C114" s="14"/>
+      <c r="D114" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="E114" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="F114" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A115" s="12"/>
+      <c r="B115" s="14"/>
+      <c r="C115" s="14"/>
+      <c r="E115" s="12"/>
+      <c r="F115" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F121" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F122" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F123" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="F124" s="8" t="s">
+        <v>212</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="L6:L7"/>
-  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1918,656 +2555,142 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G124"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="8.58203125" style="7"/>
-    <col min="2" max="2" width="22.5" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.08203125" style="17" customWidth="1"/>
-    <col min="4" max="4" width="34.83203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="35.5" style="7" customWidth="1"/>
-    <col min="6" max="6" width="48.08203125" style="9" customWidth="1"/>
-    <col min="7" max="7" width="51" style="9" customWidth="1"/>
-    <col min="8" max="16384" width="8.58203125" style="9"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="28.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.4140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="5"/>
-      <c r="B1" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="C1" s="20"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="19"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="E2" s="19"/>
-    </row>
-    <row r="4" spans="1:7" ht="17.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="11"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B5" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="13"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="13"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="8" customFormat="1" ht="51" x14ac:dyDescent="0.45">
-      <c r="A8" s="13"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="8" customFormat="1" ht="34" x14ac:dyDescent="0.45">
-      <c r="A9" s="13"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="8" customFormat="1" ht="34" x14ac:dyDescent="0.45">
-      <c r="A10" s="13"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="13"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="13"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="13"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="E13" s="13"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="D14" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="8" customFormat="1" ht="102" x14ac:dyDescent="0.45">
-      <c r="A15" s="13"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="E15" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="D17" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="D18" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="51" x14ac:dyDescent="0.45">
-      <c r="D20" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" s="23" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="21"/>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A22" s="13"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E22" s="13"/>
-      <c r="F22" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="D23" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B25" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="13"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="102" x14ac:dyDescent="0.45">
-      <c r="D27" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E27" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B31" s="17" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="34" x14ac:dyDescent="0.45">
-      <c r="D32" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E32" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="E33" s="18"/>
-    </row>
-    <row r="34" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="13"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="E34" s="13"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="D35" s="17" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="13"/>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="D37" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C39" s="17" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="13"/>
-      <c r="B40" s="15"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E40" s="13"/>
-      <c r="F40" s="8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="13"/>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="E41" s="13"/>
-      <c r="F41" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A42" s="13"/>
-      <c r="B42" s="15"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="E42" s="13"/>
-      <c r="F42" s="8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A44" s="13"/>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="E44" s="13"/>
-    </row>
-    <row r="45" spans="1:6" s="8" customFormat="1" ht="85" x14ac:dyDescent="0.45">
-      <c r="A45" s="13"/>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="E45" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C49" s="17" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="68" x14ac:dyDescent="0.45">
-      <c r="D50" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="E50" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F51" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F52" s="9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="13"/>
-      <c r="B54" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="C54" s="15"/>
-      <c r="E54" s="13"/>
-    </row>
-    <row r="55" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="13"/>
-      <c r="B55" s="15"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="E55" s="13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A57" s="13"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="E57" s="13"/>
-    </row>
-    <row r="58" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="13"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="E58" s="13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B61" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="D62" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B65" s="17" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B73" s="17" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D74" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="F74" s="8" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="I1" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="J1" s="26"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F2" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="F75" s="8" t="s">
+      <c r="G2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I2" t="s">
+        <v>271</v>
+      </c>
+      <c r="J2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B3" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D76" s="9" t="s">
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C4" t="s">
         <v>260</v>
       </c>
-      <c r="E76" s="9"/>
-    </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D77" s="9" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C5" t="s">
         <v>261</v>
       </c>
-      <c r="E77" s="9"/>
-    </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D78" s="9" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C6" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D79" s="9" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="D80" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B82" s="17" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B94" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="C94" s="24" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A95" s="13"/>
-      <c r="B95" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="C95" s="15"/>
-      <c r="D95" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="E95" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="F95" s="8" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A96" s="13"/>
-      <c r="B96" s="15"/>
-      <c r="C96" s="15"/>
-      <c r="D96" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E96" s="13"/>
-      <c r="F96" s="8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A97" s="13"/>
-      <c r="B97" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="C97" s="15"/>
-      <c r="D97" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="E97" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="F97" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A98" s="13"/>
-      <c r="B98" s="15"/>
-      <c r="C98" s="15"/>
-      <c r="D98" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="E98" s="13"/>
-      <c r="F98" s="8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B99" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="D99" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="E99" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" s="8" customFormat="1" ht="68" x14ac:dyDescent="0.45">
-      <c r="A107" s="13"/>
-      <c r="B107" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C107" s="15"/>
-      <c r="D107" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E107" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="F107" s="8" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A108" s="13"/>
-      <c r="B108" s="15"/>
-      <c r="C108" s="15"/>
-      <c r="E108" s="13"/>
-      <c r="F108" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" s="8" customFormat="1" ht="51" x14ac:dyDescent="0.45">
-      <c r="A114" s="13"/>
-      <c r="B114" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C114" s="15"/>
-      <c r="D114" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="E114" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="F114" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A115" s="13"/>
-      <c r="B115" s="15"/>
-      <c r="C115" s="15"/>
-      <c r="E115" s="13"/>
-      <c r="F115" s="8" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F121" s="9" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F122" s="9" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F123" s="9" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="F124" s="9" t="s">
-        <v>224</v>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" t="s">
+        <v>265</v>
+      </c>
+      <c r="F7" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>272</v>
+      </c>
+      <c r="F9" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>275</v>
+      </c>
+      <c r="F10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>274</v>
+      </c>
+      <c r="F11" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>278</v>
+      </c>
+      <c r="C12" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C13" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="C14" t="s">
+        <v>280</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I1:J1"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2585,46 +2708,46 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="D4" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="E4" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="F4" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="G4" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="H4" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="I4" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="C5" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="D5" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2633,23 +2756,23 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="H5" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="I5" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.45">
       <c r="G6" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2671,240 +2794,240 @@
   <sheetData>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G6" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="H6" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="I6" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="D7" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="E7" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="F7" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="G7" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="H7" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="I7" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="J7" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="F8" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="G8" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="D9" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="E9" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="F9" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="G9" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="H9" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="I9" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="J9" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="D10" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="D11" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="E11" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="F11" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="G11" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="H11" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="D12" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="E12" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="F12" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="G12" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="H12" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="I12" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="D13" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="E13" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="F13" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D14" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C15" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="F16" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="G16" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C17" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="D17" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="E17" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="F17" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="G17" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="H17" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="3:8" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="3:8" x14ac:dyDescent="0.45">
@@ -2929,42 +3052,42 @@
   <dimension ref="B2:E5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="11.75" style="25" customWidth="1"/>
+    <col min="2" max="2" width="11.75" style="24" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
     <col min="4" max="4" width="38.1640625" customWidth="1"/>
     <col min="5" max="5" width="34.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B2" s="25" t="s">
-        <v>146</v>
+      <c r="B2" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="C2" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="D2" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="E2" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B4" s="25" t="s">
-        <v>150</v>
+      <c r="B4" s="24" t="s">
+        <v>138</v>
       </c>
       <c r="C4" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="D4" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="E4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.45">
-      <c r="B5" s="25">
+      <c r="B5" s="24">
         <v>45498</v>
       </c>
     </row>

</xml_diff>